<commit_message>
Add TiSLY PLC Builder v5.10 PLC selection integration
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PLC_TEMPLATE_BUILDER/v5/generated_projects/CARSHOP_NIGHT_SECURITY/SPEC/TOMS_QUOTE.xlsx
+++ b/PLC_TEMPLATE_BUILDER/v5/generated_projects/CARSHOP_NIGHT_SECURITY/SPEC/TOMS_QUOTE.xlsx
@@ -4,6 +4,7 @@
   <sheets>
     <sheet name="見積明細" sheetId="1" r:id="rId1"/>
     <sheet name="案件情報" sheetId="2" r:id="rId2"/>
+    <sheet name="PLC容量判定" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -457,7 +458,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-30 15:36 UTC</t>
+          <t>2026-05-30 15:58 UTC</t>
         </is>
       </c>
     </row>
@@ -469,7 +470,123 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TiSLY PLC Builder v5.7</t>
+          <t>TiSLY PLC Builder v5.10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PLC型番</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FX5UJ-24MR/ES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>入力使用点数</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>8 点</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>出力使用点数</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5 点</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>入力余裕率</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>42.9 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>出力余裕率</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>50.0 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OK — 現在PLCで問題なし</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>推奨PLC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FX5UJ-24MR/ES</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>推奨拡張ユニット</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>不要</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add TiSLY PLC Builder v5.11 price estimation
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PLC_TEMPLATE_BUILDER/v5/generated_projects/CARSHOP_NIGHT_SECURITY/SPEC/TOMS_QUOTE.xlsx
+++ b/PLC_TEMPLATE_BUILDER/v5/generated_projects/CARSHOP_NIGHT_SECURITY/SPEC/TOMS_QUOTE.xlsx
@@ -11,7 +11,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -73,12 +73,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>65000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t/>
+          <t>65000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -110,12 +110,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>6500</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t/>
+          <t>6500</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>18000</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t/>
+          <t>72000</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -184,12 +184,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t/>
+          <t>6000</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t/>
+          <t>12000</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t/>
+          <t>12000</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t/>
+          <t>12000</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -258,12 +258,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>8000</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t/>
+          <t>32000</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -295,12 +295,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t/>
+          <t>3500</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t/>
+          <t>3500</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -332,17 +332,128 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t/>
+          <t>2500</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t/>
+          <t>10000</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Y1〜Y4用</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小計</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>213000</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>消費税</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>21300</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>税込合計</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>234300</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -458,7 +569,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-30 15:58 UTC</t>
+          <t>2026-05-31 00:12 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>